<commit_message>
fix(dispatcher): resolve broken cross-sheet ref in standalone earthwork dossier
Root cause: the master workbook has no Excel-cached values, so
sanitize_workbook_formulas found None for cross-sheet cells and left the
formula pointing at a sheet that does not exist in standalone files.
extract_master_eval_cache now self-evaluates missing cells via excel_eval.

Also repairs 02_Khoi_Luong_Dao_Dap_Mong_Cong_A5.xlsx (DAO_DAP!I8): the
reference to QS_DIEN_GIAI_CHI_TIET!I8 is replaced by its value 895.186
(note added in J8). Result matches the master (20804.814).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xu17UUNVqCoEvpVUxkPSc
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CONG_HOP_TUYEN_A5/BO_HO_SO_02_VI_MO_CHUYEN_SAU_14_BO/02_Khoi_Luong_Dao_Dap_Mong_Cong_A5.xlsx
+++ b/examples/HO_SO_CONG_HOP_TUYEN_A5/BO_HO_SO_02_VI_MO_CHUYEN_SAU_14_BO/02_Khoi_Luong_Dao_Dap_Mong_Cong_A5.xlsx
@@ -663,12 +663,12 @@
         <v>1</v>
       </c>
       <c r="I8" s="3">
-        <f>D8*E8*F8*G8*H8-QS_DIEN_GIAI_CHI_TIET!I8</f>
+        <f>D8*E8*F8*G8*H8-895.186</f>
         <v/>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Đầm cóc phân lớp &lt;=20cm</t>
+          <t>Đầm cóc phân lớp &lt;=20cm. Đã trừ 895.186 m3 BT thân cống đơn 2.0x2.0m (Master: QS_DIEN_GIAI_CHI_TIET!I8)</t>
         </is>
       </c>
     </row>

</xml_diff>